<commit_message>
data(pilot_006): J12(batch009 두 arm 9표본) 초안 기준 판정·검토 시트 v1(J11 같음 8/43, J12 정답 있음 Full 17·Partial 19, 우선순위 높음 39), 세션 2b GPU 큐 기록(timeline·runs·worktree 모두 지움)·사용률(utilization_s2b: GPU 0 99.6%, 1 82.5%, 2 87.8%)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017yPQTRSnHr7VQ3bAXeWQM6
</commit_message>
<xml_diff>
--- a/sft_dpo_inventory/batch009/review/batch009_review_v1.xlsx
+++ b/sft_dpo_inventory/batch009/review/batch009_review_v1.xlsx
@@ -186,7 +186,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-27</t>
+          <t xml:space="preserve">b009-21</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -201,32 +201,32 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난주 대구 중구에서 탄 손님이 많이 내린 H3 셀 세 곳을 알려줘</t>
+          <t xml:space="preserve">지난주 대구 수성구에서 손님을 태운 건수를 손님을 내려준 H3 셀별로 보여줘</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "중구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 중구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit"}], "factors": {"date": "last_week", "dimension": "h3", "dimension_target": "dropoff", "order": "top", "limit": 3}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수성구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 수성구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_week", "dimension": "h3", "dimension_target": "dropoff"}}</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 중구에서 탄 = od pickup, 많이 내린 셀 = dt dropoff + top 3.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 수성구에서 태운 = od pickup, 내려준 H3 셀별 = dt dropoff. 순위 없음.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">같음</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">3/9</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">5/9</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -236,12 +236,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t xml:space="preserve">수정(측정 span)</t>
+          <t xml:space="preserve">승인</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">질문에 측정 표현(건수)이 없어 span을 찾지 못했다. 뜻은 정답 호출과 맞지만 측정 text가 비어 학습 레코드의 측정 span이 없다. 질문에 '건수'를 넣는 수정 또는 그대로 승인(측정 text 없이)을 사람이 정한다.</t>
+          <t xml:space="preserve">정답 호출이 질문의 장소 끝(od_role)·묶는 끝(dimension_target)·묶음 단위·순위와 맞다. 검증 사슬·결정 120 겹침 검사 통과. </t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -278,7 +278,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-38</t>
+          <t xml:space="preserve">b009-22</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -293,32 +293,32 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난주 손님을 태운 셀과 내려준 셀의 짝 가운데 가장 흔한 다섯 개</t>
+          <t xml:space="preserve">이번 달 부산에서 손님이 내린 건수가 가장 적은 시군구 두 곳을 알려줘</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit"}], "factors": {"date": "last_week", "dimension": "h3", "dimension_target": "both", "order": "top", "limit": 5}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "부산"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_month", "dimension": "sigungu", "dimension_target": "dropoff", "order": "bottom", "limit": 2}}</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 태운 셀·내려준 셀 짝 = dt both(h3), 가장 흔한 다섯 개 = top 5.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 부산에서 내린 = od dropoff, 내린 시군구 기준 = dt dropoff, 가장 적은 두 곳 = bottom 2.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -328,12 +328,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t xml:space="preserve">수정(측정 span)</t>
+          <t xml:space="preserve">승인</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">질문에 측정 표현(건수)이 없어 span을 찾지 못했다. 뜻은 정답 호출과 맞지만 측정 text가 비어 학습 레코드의 측정 span이 없다. 질문에 '건수'를 넣는 수정 또는 그대로 승인(측정 text 없이)을 사람이 정한다.</t>
+          <t xml:space="preserve">정답 호출이 질문의 장소 끝(od_role)·묶는 끝(dimension_target)·묶음 단위·순위와 맞다. 검증 사슬·결정 120 겹침 검사 통과. </t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -370,12 +370,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-21</t>
+          <t xml:space="preserve">b009-23</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -385,32 +385,32 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난주 대구 수성구에서 손님을 태운 건수를 손님을 내려준 H3 셀별로 보여줘</t>
+          <t xml:space="preserve">2026년 8월 손님이 택시에 오른 건수가 가장 많은 시도 한 곳은?</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수성구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 수성구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_week", "dimension": "h3", "dimension_target": "dropoff"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "20260801-20260831", "dimension": "sido", "dimension_target": "pickup", "order": "top", "limit": 1}}</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 수성구에서 태운 = od pickup, 내려준 H3 셀별 = dt dropoff. 순위 없음.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 택시에 오른 = 승차 끝으로 묶음(dt pickup), 가장 많은 한 곳 = top 1.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -462,12 +462,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-22</t>
+          <t xml:space="preserve">b009-24</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -477,32 +477,32 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 달 부산에서 손님이 내린 건수가 가장 적은 시군구 두 곳을 알려줘</t>
+          <t xml:space="preserve">지난달 대구 동구에 손님을 내려준 건수를 손님을 태운 시도별로 세어줘</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "부산"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_month", "dimension": "sigungu", "dimension_target": "dropoff", "order": "bottom", "limit": 2}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "동구", "region": "대구"}, "attributes": {"od_role": "dropoff"}, "text": "대구 동구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_month", "dimension": "sido", "dimension_target": "pickup"}}</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 부산에서 내린 = od dropoff, 내린 시군구 기준 = dt dropoff, 가장 적은 두 곳 = bottom 2.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 동구에 내려준 = od dropoff, 태운 시도별 = dt pickup. 순위 없음.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2/9</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">6/9</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -554,12 +554,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-23</t>
+          <t xml:space="preserve">b009-27</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -569,32 +569,32 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026년 8월 손님이 택시에 오른 건수가 가장 많은 시도 한 곳은?</t>
+          <t xml:space="preserve">지난주 대구 중구에서 탄 손님이 많이 내린 H3 셀 세 곳을 알려줘</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "20260801-20260831", "dimension": "sido", "dimension_target": "pickup", "order": "top", "limit": 1}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "중구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 중구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit"}], "factors": {"date": "last_week", "dimension": "h3", "dimension_target": "dropoff", "order": "top", "limit": 3}}</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 택시에 오른 = 승차 끝으로 묶음(dt pickup), 가장 많은 한 곳 = top 1.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 중구에서 탄 = od pickup, 많이 내린 셀 = dt dropoff + top 3.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2/9</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -604,12 +604,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t xml:space="preserve">승인</t>
+          <t xml:space="preserve">수정(측정 span)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t xml:space="preserve">정답 호출이 질문의 장소 끝(od_role)·묶는 끝(dimension_target)·묶음 단위·순위와 맞다. 검증 사슬·결정 120 겹침 검사 통과. </t>
+          <t xml:space="preserve">질문에 측정 표현(건수)이 없어 span을 찾지 못했다. 뜻은 정답 호출과 맞지만 측정 text가 비어 학습 레코드의 측정 span이 없다. 질문에 '건수'를 넣는 수정 또는 그대로 승인(측정 text 없이)을 사람이 정한다.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -646,12 +646,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-24</t>
+          <t xml:space="preserve">b009-30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -661,32 +661,32 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난달 대구 동구에 손님을 내려준 건수를 손님을 태운 시도별로 세어줘</t>
+          <t xml:space="preserve">지난달 손님을 내려준 H3 셀 가운데 건수가 가장 적은 곳 하나는?</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "동구", "region": "대구"}, "attributes": {"od_role": "dropoff"}, "text": "대구 동구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_month", "dimension": "sido", "dimension_target": "pickup"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_month", "dimension": "h3", "dimension_target": "dropoff", "order": "bottom", "limit": 1}}</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 동구에 내려준 = od dropoff, 태운 시도별 = dt pickup. 순위 없음.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 내려준 셀 = dt dropoff, 가장 적은 하나 = bottom 1.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -738,12 +738,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-30</t>
+          <t xml:space="preserve">b009-33</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -753,32 +753,32 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난달 손님을 내려준 H3 셀 가운데 건수가 가장 적은 곳 하나는?</t>
+          <t xml:space="preserve">2026년 8월 대구에 내린 손님이 탄 H3 셀 가운데 건수가 많은 세 곳은?</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_month", "dimension": "h3", "dimension_target": "dropoff", "order": "bottom", "limit": 1}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "대구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "20260801-20260831", "dimension": "h3", "dimension_target": "pickup", "order": "top", "limit": 3}}</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 내려준 셀 = dt dropoff, 가장 적은 하나 = bottom 1.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 대구에 내린 = od dropoff, 탄 셀 = dt pickup, 많은 세 곳 = top 3.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -830,12 +830,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-33</t>
+          <t xml:space="preserve">b009-34</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -845,32 +845,32 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026년 8월 대구에 내린 손님이 탄 H3 셀 가운데 건수가 많은 세 곳은?</t>
+          <t xml:space="preserve">이번 주 부산 안에서만 태우고 내려준 건수를 태운 곳과 내린 곳의 시군구 짝으로 보여줘</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "대구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "20260801-20260831", "dimension": "h3", "dimension_target": "pickup", "order": "top", "limit": 3}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "pickup"}, "text": "부산"}, {"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "부산"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_week", "dimension": "sigungu", "dimension_target": "both"}}</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 대구에 내린 = od dropoff, 탄 셀 = dt pickup, 많은 세 곳 = top 3.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 부산 안에서만 태우고 내려줌 = 장소 하나 + od both, 태운 곳·내린 곳 짝 = dt both. 순위 없음.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">5/9</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">6/9</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -922,12 +922,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-34</t>
+          <t xml:space="preserve">b009-35</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -937,32 +937,32 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 주 부산 안에서만 태우고 내려준 건수를 태운 곳과 내린 곳의 시군구 짝으로 보여줘</t>
+          <t xml:space="preserve">지난달 손님이 오른 읍면동별 건수를 알려줘</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "pickup"}, "text": "부산"}, {"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "부산"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_week", "dimension": "sigungu", "dimension_target": "both"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_month", "dimension": "emd", "dimension_target": "pickup"}}</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 부산 안에서만 태우고 내려줌 = 장소 하나 + od both, 태운 곳·내린 곳 짝 = dt both. 순위 없음.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 손님이 오른 읍면동별 = dt pickup. 순위 없음.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1014,12 +1014,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-35</t>
+          <t xml:space="preserve">b009-37</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1029,32 +1029,32 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난달 손님이 오른 읍면동별 건수를 알려줘</t>
+          <t xml:space="preserve">이번 달 부산 수영구에 내려준 손님을 어느 시도에서 태웠는지 건수가 많은 곳 하나</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_month", "dimension": "emd", "dimension_target": "pickup"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수영구", "region": "부산"}, "attributes": {"od_role": "dropoff"}, "text": "부산 수영구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_month", "dimension": "sido", "dimension_target": "pickup", "order": "top", "limit": 1}}</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 손님이 오른 읍면동별 = dt pickup. 순위 없음.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 수영구에 내려준 = od dropoff, 어느 시도에서 태웠는지 = dt pickup, 많은 곳 하나 = top 1.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1106,12 +1106,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-37</t>
+          <t xml:space="preserve">b009-38</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1121,32 +1121,32 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 달 부산 수영구에 내려준 손님을 어느 시도에서 태웠는지 건수가 많은 곳 하나</t>
+          <t xml:space="preserve">지난주 손님을 태운 셀과 내려준 셀의 짝 가운데 가장 흔한 다섯 개</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수영구", "region": "부산"}, "attributes": {"od_role": "dropoff"}, "text": "부산 수영구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_month", "dimension": "sido", "dimension_target": "pickup", "order": "top", "limit": 1}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit"}], "factors": {"date": "last_week", "dimension": "h3", "dimension_target": "both", "order": "top", "limit": 5}}</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 수영구에 내려준 = od dropoff, 어느 시도에서 태웠는지 = dt pickup, 많은 곳 하나 = top 1.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 태운 셀·내려준 셀 짝 = dt both(h3), 가장 흔한 다섯 개 = top 5.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1156,12 +1156,12 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t xml:space="preserve">승인</t>
+          <t xml:space="preserve">수정(측정 span)</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t xml:space="preserve">정답 호출이 질문의 장소 끝(od_role)·묶는 끝(dimension_target)·묶음 단위·순위와 맞다. 검증 사슬·결정 120 겹침 검사 통과. </t>
+          <t xml:space="preserve">질문에 측정 표현(건수)이 없어 span을 찾지 못했다. 뜻은 정답 호출과 맞지만 측정 text가 비어 학습 레코드의 측정 span이 없다. 질문에 '건수'를 넣는 수정 또는 그대로 승인(측정 text 없이)을 사람이 정한다.</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1228,17 +1228,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1320,17 +1320,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1412,17 +1412,17 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">5/9</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1504,17 +1504,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1566,12 +1566,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-49</t>
+          <t xml:space="preserve">b009-50</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1581,32 +1581,32 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 달 대구 동구에서 승차하고 부산에서 하차한 실차 건수를 출발·도착 시군구 짝으로 보여줘</t>
+          <t xml:space="preserve">지난달 부산 수영구에서 출발한 실차 건수를 도착 H3 셀별로 많은 순 두 곳</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "동구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 동구"}, {"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "부산"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "this_month", "dimension": "sigungu", "dimension_target": "both"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수영구", "region": "부산"}, "attributes": {"od_role": "pickup"}, "text": "부산 수영구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "last_month", "dimension": "h3", "dimension_target": "dropoff", "order": "top", "limit": 2}}</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 동구 승차 = od pickup, 부산 하차 = od dropoff, 출발·도착 시군구 짝 = dt both.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 수영구 출발 = od pickup, 도착 셀별 = dt dropoff, 많은 순 두 곳 = top 2.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">7/9</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">5/9</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1658,47 +1658,47 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-50</t>
+          <t xml:space="preserve">b009-52</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">w3_od_ne_dt</t>
+          <t xml:space="preserve">w4_dt_no_rank</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난달 부산 수영구에서 출발한 실차 건수를 도착 H3 셀별로 많은 순 두 곳</t>
+          <t xml:space="preserve">이번 달 실차 건수를 승차 시군구별로 알려줘</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수영구", "region": "부산"}, "attributes": {"od_role": "pickup"}, "text": "부산 수영구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "last_month", "dimension": "h3", "dimension_target": "dropoff", "order": "top", "limit": 2}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "this_month", "dimension": "sigungu", "dimension_target": "pickup"}}</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 수영구 출발 = od pickup, 도착 셀별 = dt dropoff, 많은 순 두 곳 = top 2.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 장소 제한 없음, 승차 시군구별 = dt pickup.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2/9</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1/9</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1750,12 +1750,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-52</t>
+          <t xml:space="preserve">b009-53</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1765,32 +1765,32 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 달 실차 건수를 승차 시군구별로 알려줘</t>
+          <t xml:space="preserve">2026년 8월 실차 이동 건수를 출발 셀과 도착 셀 짝으로 정리해줘</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "this_month", "dimension": "sigungu", "dimension_target": "pickup"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 이동 건수"}], "factors": {"date": "20260801-20260831", "dimension": "h3", "dimension_target": "both"}}</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 장소 제한 없음, 승차 시군구별 = dt pickup.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 장소 제한 없음, 출발·도착 셀 짝 = dt both(h3).</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1/9</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1842,12 +1842,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-53</t>
+          <t xml:space="preserve">b009-60</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1857,32 +1857,32 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026년 8월 실차 이동 건수를 출발 셀과 도착 셀 짝으로 정리해줘</t>
+          <t xml:space="preserve">지난달 대구 안에서 승차하고 하차한 실차 건수를 승차·하차 H3 셀 짝으로 정리해줘</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 이동 건수"}], "factors": {"date": "20260801-20260831", "dimension": "h3", "dimension_target": "both"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "pickup"}, "text": "대구"}, {"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "대구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "last_month", "dimension": "h3", "dimension_target": "both"}}</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 장소 제한 없음, 출발·도착 셀 짝 = dt both(h3).</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 대구 안 승차·하차 = 장소 하나 + od both, 승차·하차 셀 짝 = dt both.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">3/9</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1/9</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1934,47 +1934,47 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-56</t>
+          <t xml:space="preserve">b009-61</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">w4_dt_no_rank</t>
+          <t xml:space="preserve">w2_implicit_endpoint_verb</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 주 대구 중구에서 출발한 실차 건수를 출발·도착 시군구 짝으로 나눠줘</t>
+          <t xml:space="preserve">이번 주 손님들이 많이 내린 H3 셀 두 곳의 건수를 알려줘</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "중구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 중구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "this_week", "dimension": "sigungu", "dimension_target": "both"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_week", "dimension": "h3", "dimension_target": "dropoff", "order": "top", "limit": 2}}</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 중구 출발 = od pickup, 출발·도착 시군구 짝 = dt both.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 많이 내린 셀 = dt dropoff + top 2.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">3/9</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">3/9</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2026,47 +2026,47 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-58</t>
+          <t xml:space="preserve">b009-62</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">w4_dt_no_rank</t>
+          <t xml:space="preserve">w2_implicit_endpoint_verb</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026년 9월 1일부터 15일까지 대구 달서구에 도착한 실차 건수를 출발·도착 H3 셀 짝으로 나눠줘</t>
+          <t xml:space="preserve">2026년 8월 손님을 태운 건수가 가장 적은 읍면동 세 곳은?</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "달서구", "region": "대구"}, "attributes": {"od_role": "dropoff"}, "text": "대구 달서구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "20260901-20260915", "dimension": "h3", "dimension_target": "both"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "20260801-20260831", "dimension": "emd", "dimension_target": "pickup", "order": "bottom", "limit": 3}}</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 달서구 도착 = od dropoff, 출발·도착 셀 짝 = dt both.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 태운 읍면동 = dt pickup, 가장 적은 세 곳 = bottom 3.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2118,47 +2118,47 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-60</t>
+          <t xml:space="preserve">b009-63</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">w4_dt_no_rank</t>
+          <t xml:space="preserve">w2_implicit_endpoint_verb</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난달 대구 안에서 승차하고 하차한 실차 건수를 승차·하차 H3 셀 짝으로 정리해줘</t>
+          <t xml:space="preserve">주말에 대구 수성구에서 손님을 태운 건수가 적은 H3 셀 두 곳</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "pickup"}, "text": "대구"}, {"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "대구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "last_month", "dimension": "h3", "dimension_target": "both"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수성구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 수성구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "weekend", "dimension": "h3", "dimension_target": "pickup", "order": "bottom", "limit": 2}}</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 대구 안 승차·하차 = 장소 하나 + od both, 승차·하차 셀 짝 = dt both.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 수성구에서 태운 = od pickup, 태운 셀 = dt pickup, 적은 두 곳 = bottom 2.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2210,12 +2210,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-61</t>
+          <t xml:space="preserve">b009-64</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2225,32 +2225,32 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 주 손님들이 많이 내린 H3 셀 두 곳의 건수를 알려줘</t>
+          <t xml:space="preserve">지난달 부산에 손님을 내려준 건수가 많은 시군구 세 곳</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_week", "dimension": "h3", "dimension_target": "dropoff", "order": "top", "limit": 2}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "부산"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_month", "dimension": "sigungu", "dimension_target": "dropoff", "order": "top", "limit": 3}}</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 많이 내린 셀 = dt dropoff + top 2.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 부산에 내려준 = od dropoff, 내려준 시군구 = dt dropoff, 많은 세 곳 = top 3.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2302,12 +2302,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-62</t>
+          <t xml:space="preserve">b009-65</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2317,32 +2317,32 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026년 8월 손님을 태운 건수가 가장 적은 읍면동 세 곳은?</t>
+          <t xml:space="preserve">이번 달 대구에 내린 손님들이 탄 셀과 내린 셀의 짝 가운데 건수가 많은 세 개</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "20260801-20260831", "dimension": "emd", "dimension_target": "pickup", "order": "bottom", "limit": 3}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "대구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_month", "dimension": "h3", "dimension_target": "both", "order": "top", "limit": 3}}</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 태운 읍면동 = dt pickup, 가장 적은 세 곳 = bottom 3.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 대구에 내린 = od dropoff, 탄 셀·내린 셀 짝 = dt both, 많은 세 개 = top 3.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -2394,12 +2394,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-63</t>
+          <t xml:space="preserve">b009-66</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2409,32 +2409,32 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">주말에 대구 수성구에서 손님을 태운 건수가 적은 H3 셀 두 곳</t>
+          <t xml:space="preserve">지난주 대구 동구에서 손님을 태운 운행을 태운 시군구와 내려준 시군구 짝으로 묶었을 때 건수가 가장 적은 두 짝</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수성구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 수성구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "weekend", "dimension": "h3", "dimension_target": "pickup", "order": "bottom", "limit": 2}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "동구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 동구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_week", "dimension": "sigungu", "dimension_target": "both", "order": "bottom", "limit": 2}}</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 수성구에서 태운 = od pickup, 태운 셀 = dt pickup, 적은 두 곳 = bottom 2.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 동구에서 태운 = od pickup, 태운·내려준 시군구 짝 = dt both, 가장 적은 두 짝 = bottom 2.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1/9</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -2486,12 +2486,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-64</t>
+          <t xml:space="preserve">b009-67</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2501,32 +2501,32 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난달 부산에 손님을 내려준 건수가 많은 시군구 세 곳</t>
+          <t xml:space="preserve">이번 주 부산 수영구에 손님을 내려준 건수를 태운 읍면동과 내려준 읍면동 짝으로 보면 가장 흔한 세 짝은?</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "부산"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_month", "dimension": "sigungu", "dimension_target": "dropoff", "order": "top", "limit": 3}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수영구", "region": "부산"}, "attributes": {"od_role": "dropoff"}, "text": "부산 수영구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_week", "dimension": "emd", "dimension_target": "both", "order": "top", "limit": 3}}</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 부산에 내려준 = od dropoff, 내려준 시군구 = dt dropoff, 많은 세 곳 = top 3.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 수영구에 내려준 = od dropoff, 태운·내려준 읍면동 짝 = dt both, 가장 흔한 세 짝 = top 3.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">같음</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2578,12 +2578,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-65</t>
+          <t xml:space="preserve">b009-68</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2593,32 +2593,32 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 달 대구에 내린 손님들이 탄 셀과 내린 셀의 짝 가운데 건수가 많은 세 개</t>
+          <t xml:space="preserve">지난달 대구 안에서 태워 대구 안에 내려준 건수가 많은 태운 셀 세 곳</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "대구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_month", "dimension": "h3", "dimension_target": "both", "order": "top", "limit": 3}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "pickup"}, "text": "대구"}, {"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "대구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_month", "dimension": "h3", "dimension_target": "pickup", "order": "top", "limit": 3}}</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 대구에 내린 = od dropoff, 탄 셀·내린 셀 짝 = dt both, 많은 세 개 = top 3.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 대구 안에서 태워 대구 안에 내려줌 = 장소 하나 + od both, 태운 셀 = dt pickup, 많은 세 곳 = top 3.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2670,12 +2670,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-66</t>
+          <t xml:space="preserve">b009-69</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2685,32 +2685,32 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난주 대구 동구에서 손님을 태운 운행을 태운 시군구와 내려준 시군구 짝으로 묶었을 때 건수가 가장 적은 두 짝</t>
+          <t xml:space="preserve">주말 대구 수성구에서 태워 부산에 내려준 건수가 적은 태운 셀 두 곳</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "동구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 동구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_week", "dimension": "sigungu", "dimension_target": "both", "order": "bottom", "limit": 2}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수성구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 수성구"}, {"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "부산"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "weekend", "dimension": "h3", "dimension_target": "pickup", "order": "bottom", "limit": 2}}</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 동구에서 태운 = od pickup, 태운·내려준 시군구 짝 = dt both, 가장 적은 두 짝 = bottom 2.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 수성구에서 태움 = od pickup, 부산에 내려줌 = od dropoff, 태운 셀 = dt pickup, 적은 두 곳 = bottom 2.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2762,12 +2762,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-67</t>
+          <t xml:space="preserve">b009-70</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2777,32 +2777,32 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 주 부산 수영구에 손님을 내려준 건수를 태운 읍면동과 내려준 읍면동 짝으로 보면 가장 흔한 세 짝은?</t>
+          <t xml:space="preserve">이번 달 손님을 내려준 건수가 가장 적은 시도 한 곳</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수영구", "region": "부산"}, "attributes": {"od_role": "dropoff"}, "text": "부산 수영구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_week", "dimension": "emd", "dimension_target": "both", "order": "top", "limit": 3}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_month", "dimension": "sido", "dimension_target": "dropoff", "order": "bottom", "limit": 1}}</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 수영구에 내려준 = od dropoff, 태운·내려준 읍면동 짝 = dt both, 가장 흔한 세 짝 = top 3.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 내려준 시도 = dt dropoff, 가장 적은 한 곳 = bottom 1.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2/9</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2854,12 +2854,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-68</t>
+          <t xml:space="preserve">b009-71</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2869,32 +2869,32 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난달 대구 안에서 태워 대구 안에 내려준 건수가 많은 태운 셀 세 곳</t>
+          <t xml:space="preserve">지난달 부산진구에 내려준 손님을 태운 시도 가운데 건수가 가장 적은 곳</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "pickup"}, "text": "대구"}, {"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "대구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_month", "dimension": "h3", "dimension_target": "pickup", "order": "top", "limit": 3}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산진구", "region": "부산"}, "attributes": {"od_role": "dropoff"}, "text": "부산진구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_month", "dimension": "sido", "dimension_target": "pickup", "order": "bottom", "limit": 1}}</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 대구 안에서 태워 대구 안에 내려줌 = 장소 하나 + od both, 태운 셀 = dt pickup, 많은 세 곳 = top 3.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 부산진구에 내려준 = od dropoff, 태운 시도 = dt pickup, 가장 적은 곳 = bottom 1.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2946,12 +2946,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-69</t>
+          <t xml:space="preserve">b009-72</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2961,32 +2961,32 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">주말 대구 수성구에서 태워 부산에 내려준 건수가 적은 태운 셀 두 곳</t>
+          <t xml:space="preserve">이번 주 대구 달서구에서 손님을 태운 건수를 태운 셀과 내려준 셀 짝으로 많은 순 세 개</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수성구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 수성구"}, {"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "부산"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "weekend", "dimension": "h3", "dimension_target": "pickup", "order": "bottom", "limit": 2}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "달서구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 달서구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_week", "dimension": "h3", "dimension_target": "both", "order": "top", "limit": 3}}</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 수성구에서 태움 = od pickup, 부산에 내려줌 = od dropoff, 태운 셀 = dt pickup, 적은 두 곳 = bottom 2.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 달서구에서 태운 = od pickup, 태운 셀·내려준 셀 짝 = dt both, 많은 순 세 개 = top 3.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3038,47 +3038,47 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-70</t>
+          <t xml:space="preserve">b009-73</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">w2_implicit_endpoint_verb</t>
+          <t xml:space="preserve">w3_od_ne_dt</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 달 손님을 내려준 건수가 가장 적은 시도 한 곳</t>
+          <t xml:space="preserve">이번 달 대구 동구에서 승차한 실차 건수를 하차 시도별로 적은 순 한 곳</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_month", "dimension": "sido", "dimension_target": "dropoff", "order": "bottom", "limit": 1}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "동구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 동구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "this_month", "dimension": "sido", "dimension_target": "dropoff", "order": "bottom", "limit": 1}}</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 장소 제한 없음, 내려준 시도 = dt dropoff, 가장 적은 한 곳 = bottom 1.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 동구 승차 = od pickup, 하차 시도별 = dt dropoff, 적은 순 한 곳 = bottom 1.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3130,47 +3130,47 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-71</t>
+          <t xml:space="preserve">b009-75</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">w2_implicit_endpoint_verb</t>
+          <t xml:space="preserve">w3_od_ne_dt</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난달 부산진구에 내려준 손님을 태운 시도 가운데 건수가 가장 적은 곳</t>
+          <t xml:space="preserve">2026년 8월 부산 수영구에 도착한 실차 건수를 출발 H3 셀별로 많은 순 세 곳</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산진구", "region": "부산"}, "attributes": {"od_role": "dropoff"}, "text": "부산진구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "last_month", "dimension": "sido", "dimension_target": "pickup", "order": "bottom", "limit": 1}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수영구", "region": "부산"}, "attributes": {"od_role": "dropoff"}, "text": "부산 수영구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "20260801-20260831", "dimension": "h3", "dimension_target": "pickup", "order": "top", "limit": 3}}</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 부산진구에 내려준 = od dropoff, 태운 시도 = dt pickup, 가장 적은 곳 = bottom 1.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 수영구 도착 = od dropoff, 출발 셀별 = dt pickup, 많은 순 세 곳 = top 3.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -3222,47 +3222,47 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-72</t>
+          <t xml:space="preserve">b009-76</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">w2_implicit_endpoint_verb</t>
+          <t xml:space="preserve">w3_od_ne_dt</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 주 대구 달서구에서 손님을 태운 건수를 태운 셀과 내려준 셀 짝으로 많은 순 세 개</t>
+          <t xml:space="preserve">이번 주 부산진구에서 출발한 실차 건수를 출발·도착 시군구 짝으로 정리해줘</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "달서구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 달서구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "건수"}], "factors": {"date": "this_week", "dimension": "h3", "dimension_target": "both", "order": "top", "limit": 3}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산진구", "region": "부산"}, "attributes": {"od_role": "pickup"}, "text": "부산진구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "this_week", "dimension": "sigungu", "dimension_target": "both"}}</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 승차·하차·출발·도착이라는 말 없이 동사로 끝을 말한다(태운·탄·오른 = 승차 끝, 내려준·내린 = 하차 끝). 달서구에서 태운 = od pickup, 태운 셀·내려준 셀 짝 = dt both, 많은 순 세 개 = top 3.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 부산진구 출발 = od pickup, 출발·도착 시군구 짝 = dt both.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">7/9</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -3314,12 +3314,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-73</t>
+          <t xml:space="preserve">b009-77</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3329,32 +3329,32 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 달 대구 동구에서 승차한 실차 건수를 하차 시도별로 적은 순 한 곳</t>
+          <t xml:space="preserve">지난달 대구 중구에 도착한 실차 건수를 출발·도착 시군구 짝 가운데 적은 순 두 개</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "동구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 동구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "this_month", "dimension": "sido", "dimension_target": "dropoff", "order": "bottom", "limit": 1}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "중구", "region": "대구"}, "attributes": {"od_role": "dropoff"}, "text": "대구 중구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "last_month", "dimension": "sigungu", "dimension_target": "both", "order": "bottom", "limit": 2}}</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 동구 승차 = od pickup, 하차 시도별 = dt dropoff, 적은 순 한 곳 = bottom 1.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 중구 도착 = od dropoff, 출발·도착 시군구 짝 = dt both, 적은 순 두 개 = bottom 2.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">5/9</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">6/9</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -3406,47 +3406,47 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-74</t>
+          <t xml:space="preserve">b009-79</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">w3_od_ne_dt</t>
+          <t xml:space="preserve">w4_dt_no_rank</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난주 대구 수성구에서 하차한 실차 건수를 승차 읍면동별로 보여줘</t>
+          <t xml:space="preserve">2026년 9월 실차 건수를 하차 시군구별로 보여줘</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수성구", "region": "대구"}, "attributes": {"od_role": "dropoff"}, "text": "대구 수성구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "last_week", "dimension": "emd", "dimension_target": "pickup"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "20260901-20260930", "dimension": "sigungu", "dimension_target": "dropoff"}}</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 수성구 하차 = od dropoff, 승차 읍면동별 = dt pickup.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 장소 제한 없음, 하차 시군구별 = dt dropoff.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0/9</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -3498,47 +3498,47 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-75</t>
+          <t xml:space="preserve">b009-80</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">w3_od_ne_dt</t>
+          <t xml:space="preserve">w4_dt_no_rank</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026년 8월 부산 수영구에 도착한 실차 건수를 출발 H3 셀별로 많은 순 세 곳</t>
+          <t xml:space="preserve">지난주 실차 이동 건수를 출발·도착 읍면동 짝으로 정리해줘</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수영구", "region": "부산"}, "attributes": {"od_role": "dropoff"}, "text": "부산 수영구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "20260801-20260831", "dimension": "h3", "dimension_target": "pickup", "order": "top", "limit": 3}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 이동 건수"}], "factors": {"date": "last_week", "dimension": "emd", "dimension_target": "both"}}</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 수영구 도착 = od dropoff, 출발 셀별 = dt pickup, 많은 순 세 곳 = top 3.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 장소 제한 없음, 출발·도착 읍면동 짝 = dt both.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">다름</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1/9</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1/9</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -3590,47 +3590,47 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-76</t>
+          <t xml:space="preserve">b009-83</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">w3_od_ne_dt</t>
+          <t xml:space="preserve">w4_dt_no_rank</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 주 부산진구에서 출발한 실차 건수를 출발·도착 시군구 짝으로 정리해줘</t>
+          <t xml:space="preserve">주말 대구 수성구에서 출발해 부산에 도착한 실차 건수를 출발·도착 시군구 짝으로 보여줘</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산진구", "region": "부산"}, "attributes": {"od_role": "pickup"}, "text": "부산진구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "this_week", "dimension": "sigungu", "dimension_target": "both"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수성구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 수성구"}, {"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "부산"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "weekend", "dimension": "sigungu", "dimension_target": "both"}}</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 부산진구 출발 = od pickup, 출발·도착 시군구 짝 = dt both.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 수성구 출발 = od pickup, 부산 도착 = od dropoff, 출발·도착 시군구 짝 = dt both.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">같음</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">5/9</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">3/9</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3682,47 +3682,47 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-77</t>
+          <t xml:space="preserve">b009-84</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">보통</t>
+          <t xml:space="preserve">높음</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">w3_od_ne_dt</t>
+          <t xml:space="preserve">w4_dt_no_rank</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난달 대구 중구에 도착한 실차 건수를 출발·도착 시군구 짝 가운데 적은 순 두 개</t>
+          <t xml:space="preserve">이번 주 대구에서 출발한 실차 건수를 출발 시군구별로 보여줘</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "중구", "region": "대구"}, "attributes": {"od_role": "dropoff"}, "text": "대구 중구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "last_month", "dimension": "sigungu", "dimension_target": "both", "order": "bottom", "limit": 2}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "pickup"}, "text": "대구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "this_week", "dimension": "sigungu", "dimension_target": "pickup"}}</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 중구 도착 = od dropoff, 출발·도착 시군구 짝 = dt both, 적은 순 두 개 = bottom 2.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 대구 출발 = od pickup, 출발 시군구별 = dt pickup.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">같음</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2/9</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">1/9</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -3774,7 +3774,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-79</t>
+          <t xml:space="preserve">b009-49</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3784,37 +3784,37 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">w4_dt_no_rank</t>
+          <t xml:space="preserve">w3_od_ne_dt</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026년 9월 실차 건수를 하차 시군구별로 보여줘</t>
+          <t xml:space="preserve">이번 달 대구 동구에서 승차하고 부산에서 하차한 실차 건수를 출발·도착 시군구 짝으로 보여줘</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "20260901-20260930", "dimension": "sigungu", "dimension_target": "dropoff"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "동구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 동구"}, {"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "부산"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "this_month", "dimension": "sigungu", "dimension_target": "both"}}</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 장소 제한 없음, 하차 시군구별 = dt dropoff.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 동구 승차 = od pickup, 부산 하차 = od dropoff, 출발·도착 시군구 짝 = dt both.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">같음</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">4/9</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">4/9</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-80</t>
+          <t xml:space="preserve">b009-56</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3881,32 +3881,32 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">지난주 실차 이동 건수를 출발·도착 읍면동 짝으로 정리해줘</t>
+          <t xml:space="preserve">이번 주 대구 중구에서 출발한 실차 건수를 출발·도착 시군구 짝으로 나눠줘</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 이동 건수"}], "factors": {"date": "last_week", "dimension": "emd", "dimension_target": "both"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "중구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 중구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "this_week", "dimension": "sigungu", "dimension_target": "both"}}</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 장소 제한 없음, 출발·도착 읍면동 짝 = dt both.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 중구 출발 = od pickup, 출발·도착 시군구 짝 = dt both.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">같음</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">5/9</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">7/9</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -3958,7 +3958,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-83</t>
+          <t xml:space="preserve">b009-58</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3973,32 +3973,32 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">주말 대구 수성구에서 출발해 부산에 도착한 실차 건수를 출발·도착 시군구 짝으로 보여줘</t>
+          <t xml:space="preserve">2026년 9월 1일부터 15일까지 대구 달서구에 도착한 실차 건수를 출발·도착 H3 셀 짝으로 나눠줘</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수성구", "region": "대구"}, "attributes": {"od_role": "pickup"}, "text": "대구 수성구"}, {"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "부산", "region": ""}, "attributes": {"od_role": "dropoff"}, "text": "부산"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "weekend", "dimension": "sigungu", "dimension_target": "both"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "달서구", "region": "대구"}, "attributes": {"od_role": "dropoff"}, "text": "대구 달서구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "20260901-20260915", "dimension": "h3", "dimension_target": "both"}}</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 수성구 출발 = od pickup, 부산 도착 = od dropoff, 출발·도착 시군구 짝 = dt both.</t>
+          <t xml:space="preserve">실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 달서구 도착 = od dropoff, 출발·도착 셀 짝 = dt both.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">같음</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">7/9</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">4/9</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4050,7 +4050,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">b009-84</t>
+          <t xml:space="preserve">b009-74</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4060,37 +4060,37 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">w4_dt_no_rank</t>
+          <t xml:space="preserve">w3_od_ne_dt</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 주 대구에서 출발한 실차 건수를 출발 시군구별로 보여줘</t>
+          <t xml:space="preserve">지난주 대구 수성구에서 하차한 실차 건수를 승차 읍면동별로 보여줘</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">{"concepts": [{"id": "place_scope_pickup", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "대구", "region": ""}, "attributes": {"od_role": "pickup"}, "text": "대구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "this_week", "dimension": "sigungu", "dimension_target": "pickup"}}</t>
+          <t xml:space="preserve">{"concepts": [{"id": "place_scope_dropoff", "concept": "LOCATION", "subtype": "place", "role": "SUBCOND", "source": "user", "value": {"name": "수성구", "region": "대구"}, "attributes": {"od_role": "dropoff"}, "text": "대구 수성구"}, {"id": "event", "concept": "EVENT", "subtype": "trip", "role": "SUPPORT", "source": "implicit"}, {"id": "measure", "concept": "AMOUNT", "subtype": "trip_count", "role": "MEASURE", "source": "implicit", "text": "실차 건수"}], "factors": {"date": "last_week", "dimension": "emd", "dimension_target": "pickup"}}</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 순위·개수 제한이 없으므로 order·limit 없음. 대구 출발 = od pickup, 출발 시군구별 = dt pickup.</t>
+          <t xml:space="preserve">2차 후보: 1차에서 보호 넷 family·현재 코드 거부로 빠진 만큼 다시 썼다(구조는 free_structures.json의 free). 실차 건수(trip_count). 장소가 제한하는 끝 = od_role, 결과를 묶는 끝 = dimension_target. 장소가 제한하는 끝과 묶는 끝이 다르다. 수성구 하차 = od dropoff, 승차 읍면동별 = dt pickup.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">같음</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">4/9</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">5/9</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">

</xml_diff>